<commit_message>
feat(excel): refactor validation model to use declarative checks and improve import parsing
Replace inline schema validation attributes (mandatory, min, max, pattern, etc.) with a flexible `<checks>` element model supporting reusable validation rules (notNull, range, number, pattern, chinese, etc.). Refactor PoExcelHelper to use ImportExcelParser with aggregated runtime error reporting. Add tagSet-based property filtering for import/export scope control.
</commit_message>
<xml_diff>
--- a/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test-check.xlsx
+++ b/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test-check.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13404" windowHeight="4452"/>
+    <workbookView windowWidth="21000" windowHeight="4452"/>
   </bookViews>
   <sheets>
     <sheet name="TestEntity" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>唯一标识</t>
   </si>
@@ -56,9 +56,6 @@
     <t>1001</t>
   </si>
   <si>
-    <t>张三</t>
-  </si>
-  <si>
     <t>男</t>
   </si>
   <si>
@@ -68,7 +65,7 @@
     <t>1002</t>
   </si>
   <si>
-    <t>李四</t>
+    <t>lisi</t>
   </si>
   <si>
     <t>PDM</t>
@@ -90,7 +87,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <b/>
       <sz val="11"/>
@@ -107,12 +104,6 @@
       <b/>
       <sz val="11"/>
       <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -582,163 +573,160 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1100,17 +1088,15 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4">
+        <v>17</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="D4" s="3">
-        <v>17</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -1118,19 +1104,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>61</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="3">
-        <v>61</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="F5">
         <v>2</v>
@@ -1138,19 +1124,19 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>34</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="D6" s="3">
-        <v>34</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="F6">
         <v>3</v>

</xml_diff>